<commit_message>
chore(weekly-sync): auto-pull through 2026-09-07
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week36.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week36.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SB" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SB" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -494,10 +494,10 @@
         <v>7215</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>3099.16</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -662,10 +662,10 @@
         <v>53795</v>
       </c>
       <c r="G8" t="n">
-        <v>19062.7</v>
+        <v>21434.74</v>
       </c>
       <c r="H8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -690,10 +690,10 @@
         <v>16819</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>7626.27</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -827,7 +827,7 @@
         <v>315</v>
       </c>
       <c r="F14" t="n">
-        <v>34686</v>
+        <v>34684</v>
       </c>
       <c r="G14" t="n">
         <v>26968.65</v>
@@ -855,13 +855,13 @@
         <v>1150</v>
       </c>
       <c r="F15" t="n">
-        <v>70142</v>
+        <v>70141</v>
       </c>
       <c r="G15" t="n">
         <v>47329.62</v>
       </c>
       <c r="H15" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16">
@@ -886,10 +886,10 @@
         <v>1259</v>
       </c>
       <c r="G16" t="n">
-        <v>14859.31</v>
+        <v>17146.6</v>
       </c>
       <c r="H16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -1029,7 +1029,7 @@
         <v>32875.43</v>
       </c>
       <c r="H21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22">
@@ -1107,7 +1107,7 @@
         <v>1390</v>
       </c>
       <c r="F24" t="n">
-        <v>118242</v>
+        <v>118241</v>
       </c>
       <c r="G24" t="n">
         <v>83626.28</v>
@@ -1191,7 +1191,7 @@
         <v>169</v>
       </c>
       <c r="F27" t="n">
-        <v>40361</v>
+        <v>40360</v>
       </c>
       <c r="G27" t="n">
         <v>10589</v>
@@ -1219,7 +1219,7 @@
         <v>101</v>
       </c>
       <c r="F28" t="n">
-        <v>17410</v>
+        <v>17407</v>
       </c>
       <c r="G28" t="n">
         <v>2117.8</v>
@@ -1334,10 +1334,10 @@
         <v>11297</v>
       </c>
       <c r="G32" t="n">
-        <v>27452.52</v>
+        <v>41178.78</v>
       </c>
       <c r="H32" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33">
@@ -1387,7 +1387,7 @@
         <v>613</v>
       </c>
       <c r="F34" t="n">
-        <v>86034</v>
+        <v>86033</v>
       </c>
       <c r="G34" t="n">
         <v>38131.35000000001</v>
@@ -1443,7 +1443,7 @@
         <v>800</v>
       </c>
       <c r="F36" t="n">
-        <v>143317</v>
+        <v>143313</v>
       </c>
       <c r="G36" t="n">
         <v>11168.63</v>
@@ -1555,7 +1555,7 @@
         <v>666</v>
       </c>
       <c r="F40" t="n">
-        <v>54625</v>
+        <v>54624</v>
       </c>
       <c r="G40" t="n">
         <v>17273.7</v>
@@ -1695,7 +1695,7 @@
         <v>512</v>
       </c>
       <c r="F45" t="n">
-        <v>42383</v>
+        <v>42382</v>
       </c>
       <c r="G45" t="n">
         <v>2965.25</v>
@@ -1891,7 +1891,7 @@
         <v>97</v>
       </c>
       <c r="F52" t="n">
-        <v>17933</v>
+        <v>17932</v>
       </c>
       <c r="G52" t="n">
         <v>3388.13</v>
@@ -1919,7 +1919,7 @@
         <v>311</v>
       </c>
       <c r="F53" t="n">
-        <v>50563</v>
+        <v>50562</v>
       </c>
       <c r="G53" t="n">
         <v>16766.09</v>
@@ -1947,7 +1947,7 @@
         <v>21</v>
       </c>
       <c r="F54" t="n">
-        <v>10013</v>
+        <v>10010</v>
       </c>
       <c r="G54" t="n">
         <v>4236.44</v>
@@ -1975,7 +1975,7 @@
         <v>230</v>
       </c>
       <c r="F55" t="n">
-        <v>39498</v>
+        <v>39494</v>
       </c>
       <c r="G55" t="n">
         <v>3194.07</v>
@@ -2003,7 +2003,7 @@
         <v>47</v>
       </c>
       <c r="F56" t="n">
-        <v>8008</v>
+        <v>8007</v>
       </c>
       <c r="G56" t="n">
         <v>1439.83</v>
@@ -2031,7 +2031,7 @@
         <v>25</v>
       </c>
       <c r="F57" t="n">
-        <v>5754</v>
+        <v>5752</v>
       </c>
       <c r="G57" t="n">
         <v>0</v>
@@ -2059,7 +2059,7 @@
         <v>273</v>
       </c>
       <c r="F58" t="n">
-        <v>68573</v>
+        <v>68571</v>
       </c>
       <c r="G58" t="n">
         <v>8508.49</v>
@@ -2087,7 +2087,7 @@
         <v>101</v>
       </c>
       <c r="F59" t="n">
-        <v>24815</v>
+        <v>24814</v>
       </c>
       <c r="G59" t="n">
         <v>4401.700000000001</v>
@@ -2115,7 +2115,7 @@
         <v>45</v>
       </c>
       <c r="F60" t="n">
-        <v>10498</v>
+        <v>10497</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
@@ -2137,13 +2137,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>311.21</v>
+        <v>308.07</v>
       </c>
       <c r="E61" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F61" t="n">
-        <v>20075</v>
+        <v>20073</v>
       </c>
       <c r="G61" t="n">
         <v>550</v>
@@ -2199,7 +2199,7 @@
         <v>127</v>
       </c>
       <c r="F63" t="n">
-        <v>17807</v>
+        <v>17806</v>
       </c>
       <c r="G63" t="n">
         <v>3455.93</v>
@@ -2227,7 +2227,7 @@
         <v>55</v>
       </c>
       <c r="F64" t="n">
-        <v>7167</v>
+        <v>7165</v>
       </c>
       <c r="G64" t="n">
         <v>2624.58</v>
@@ -2255,7 +2255,7 @@
         <v>73</v>
       </c>
       <c r="F65" t="n">
-        <v>15044</v>
+        <v>15042</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
@@ -2283,7 +2283,7 @@
         <v>92</v>
       </c>
       <c r="F66" t="n">
-        <v>11885</v>
+        <v>11882</v>
       </c>
       <c r="G66" t="n">
         <v>1694.07</v>
@@ -2395,7 +2395,7 @@
         <v>426</v>
       </c>
       <c r="F70" t="n">
-        <v>80240</v>
+        <v>80222</v>
       </c>
       <c r="G70" t="n">
         <v>6438.98</v>
@@ -2423,7 +2423,7 @@
         <v>160</v>
       </c>
       <c r="F71" t="n">
-        <v>13182</v>
+        <v>13180</v>
       </c>
       <c r="G71" t="n">
         <v>13088.98</v>
@@ -2479,7 +2479,7 @@
         <v>195</v>
       </c>
       <c r="F73" t="n">
-        <v>39823</v>
+        <v>39821</v>
       </c>
       <c r="G73" t="n">
         <v>4778.78</v>
@@ -2507,7 +2507,7 @@
         <v>246</v>
       </c>
       <c r="F74" t="n">
-        <v>25792</v>
+        <v>25791</v>
       </c>
       <c r="G74" t="n">
         <v>2243.21</v>
@@ -2535,7 +2535,7 @@
         <v>570</v>
       </c>
       <c r="F75" t="n">
-        <v>127764</v>
+        <v>127755</v>
       </c>
       <c r="G75" t="n">
         <v>12539.82</v>
@@ -2563,13 +2563,13 @@
         <v>1713</v>
       </c>
       <c r="F76" t="n">
-        <v>259088</v>
+        <v>259076</v>
       </c>
       <c r="G76" t="n">
-        <v>17704.23</v>
+        <v>18508.47</v>
       </c>
       <c r="H76" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77">
@@ -2591,7 +2591,7 @@
         <v>36</v>
       </c>
       <c r="F77" t="n">
-        <v>17812</v>
+        <v>17811</v>
       </c>
       <c r="G77" t="n">
         <v>1007.63</v>
@@ -2619,7 +2619,7 @@
         <v>22</v>
       </c>
       <c r="F78" t="n">
-        <v>4181</v>
+        <v>4179</v>
       </c>
       <c r="G78" t="n">
         <v>0</v>
@@ -2647,7 +2647,7 @@
         <v>27</v>
       </c>
       <c r="F79" t="n">
-        <v>2499</v>
+        <v>2497</v>
       </c>
       <c r="G79" t="n">
         <v>0</v>
@@ -2675,7 +2675,7 @@
         <v>53</v>
       </c>
       <c r="F80" t="n">
-        <v>11532</v>
+        <v>11530</v>
       </c>
       <c r="G80" t="n">
         <v>0</v>
@@ -2703,7 +2703,7 @@
         <v>54</v>
       </c>
       <c r="F81" t="n">
-        <v>6934</v>
+        <v>6933</v>
       </c>
       <c r="G81" t="n">
         <v>0</v>
@@ -2759,7 +2759,7 @@
         <v>74</v>
       </c>
       <c r="F83" t="n">
-        <v>10682</v>
+        <v>10680</v>
       </c>
       <c r="G83" t="n">
         <v>6608.469999999999</v>
@@ -2787,7 +2787,7 @@
         <v>158</v>
       </c>
       <c r="F84" t="n">
-        <v>19788</v>
+        <v>19786</v>
       </c>
       <c r="G84" t="n">
         <v>10166.94</v>
@@ -2815,7 +2815,7 @@
         <v>15</v>
       </c>
       <c r="F85" t="n">
-        <v>3341</v>
+        <v>3339</v>
       </c>
       <c r="G85" t="n">
         <v>0</v>
@@ -2843,7 +2843,7 @@
         <v>606</v>
       </c>
       <c r="F86" t="n">
-        <v>79859</v>
+        <v>79858</v>
       </c>
       <c r="G86" t="n">
         <v>9308.52</v>
@@ -2871,7 +2871,7 @@
         <v>21</v>
       </c>
       <c r="F87" t="n">
-        <v>2418</v>
+        <v>2417</v>
       </c>
       <c r="G87" t="n">
         <v>2414.41</v>
@@ -2899,7 +2899,7 @@
         <v>512</v>
       </c>
       <c r="F88" t="n">
-        <v>98249</v>
+        <v>98247</v>
       </c>
       <c r="G88" t="n">
         <v>11604.25</v>
@@ -2927,7 +2927,7 @@
         <v>297</v>
       </c>
       <c r="F89" t="n">
-        <v>46758</v>
+        <v>46755</v>
       </c>
       <c r="G89" t="n">
         <v>23383.87</v>
@@ -2955,7 +2955,7 @@
         <v>49</v>
       </c>
       <c r="F90" t="n">
-        <v>6288</v>
+        <v>6287</v>
       </c>
       <c r="G90" t="n">
         <v>4490.68</v>
@@ -2983,7 +2983,7 @@
         <v>191</v>
       </c>
       <c r="F91" t="n">
-        <v>44891</v>
+        <v>44889</v>
       </c>
       <c r="G91" t="n">
         <v>21269.5</v>
@@ -3067,7 +3067,7 @@
         <v>38</v>
       </c>
       <c r="F94" t="n">
-        <v>11122</v>
+        <v>11120</v>
       </c>
       <c r="G94" t="n">
         <v>0</v>
@@ -3123,7 +3123,7 @@
         <v>92</v>
       </c>
       <c r="F96" t="n">
-        <v>20485</v>
+        <v>20484</v>
       </c>
       <c r="G96" t="n">
         <v>10294.06</v>
@@ -3151,7 +3151,7 @@
         <v>27</v>
       </c>
       <c r="F97" t="n">
-        <v>5220</v>
+        <v>5219</v>
       </c>
       <c r="G97" t="n">
         <v>0</v>
@@ -3257,19 +3257,19 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>3124.53</v>
+        <v>3123.27</v>
       </c>
       <c r="E101" t="n">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="F101" t="n">
-        <v>83666</v>
+        <v>83664</v>
       </c>
       <c r="G101" t="n">
-        <v>16649.15</v>
+        <v>22071.18</v>
       </c>
       <c r="H101" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="102">
@@ -3375,7 +3375,7 @@
         <v>24</v>
       </c>
       <c r="F105" t="n">
-        <v>4679</v>
+        <v>4678</v>
       </c>
       <c r="G105" t="n">
         <v>2172.88</v>
@@ -3403,7 +3403,7 @@
         <v>2077</v>
       </c>
       <c r="F106" t="n">
-        <v>263551</v>
+        <v>263548</v>
       </c>
       <c r="G106" t="n">
         <v>37704.23</v>
@@ -3431,13 +3431,13 @@
         <v>46</v>
       </c>
       <c r="F107" t="n">
-        <v>14335</v>
+        <v>14334</v>
       </c>
       <c r="G107" t="n">
         <v>0</v>
       </c>
       <c r="H107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -3462,10 +3462,10 @@
         <v>54967</v>
       </c>
       <c r="G108" t="n">
-        <v>26688.11</v>
+        <v>31348.28</v>
       </c>
       <c r="H108" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="109">
@@ -3543,7 +3543,7 @@
         <v>275</v>
       </c>
       <c r="F111" t="n">
-        <v>40056</v>
+        <v>40055</v>
       </c>
       <c r="G111" t="n">
         <v>21607.62</v>
@@ -3571,7 +3571,7 @@
         <v>359</v>
       </c>
       <c r="F112" t="n">
-        <v>42875</v>
+        <v>42874</v>
       </c>
       <c r="G112" t="n">
         <v>13981.35</v>
@@ -3739,7 +3739,7 @@
         <v>473</v>
       </c>
       <c r="F118" t="n">
-        <v>38887</v>
+        <v>38886</v>
       </c>
       <c r="G118" t="n">
         <v>44486.44</v>
@@ -3770,10 +3770,10 @@
         <v>65799</v>
       </c>
       <c r="G119" t="n">
-        <v>39353.4</v>
+        <v>41640.69</v>
       </c>
       <c r="H119" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="120">
@@ -3823,7 +3823,7 @@
         <v>296</v>
       </c>
       <c r="F121" t="n">
-        <v>68543</v>
+        <v>68542</v>
       </c>
       <c r="G121" t="n">
         <v>8974.57</v>
@@ -3907,7 +3907,7 @@
         <v>149</v>
       </c>
       <c r="F124" t="n">
-        <v>16317</v>
+        <v>16316</v>
       </c>
       <c r="G124" t="n">
         <v>13723.74</v>
@@ -4103,7 +4103,7 @@
         <v>857</v>
       </c>
       <c r="F131" t="n">
-        <v>86815</v>
+        <v>86813</v>
       </c>
       <c r="G131" t="n">
         <v>26690.7</v>
@@ -4187,7 +4187,7 @@
         <v>146</v>
       </c>
       <c r="F134" t="n">
-        <v>58641</v>
+        <v>58640</v>
       </c>
       <c r="G134" t="n">
         <v>13047.44</v>
@@ -4327,7 +4327,7 @@
         <v>205</v>
       </c>
       <c r="F139" t="n">
-        <v>66937</v>
+        <v>66936</v>
       </c>
       <c r="G139" t="n">
         <v>2414.41</v>
@@ -4383,7 +4383,7 @@
         <v>97</v>
       </c>
       <c r="F141" t="n">
-        <v>37495</v>
+        <v>37492</v>
       </c>
       <c r="G141" t="n">
         <v>5930.5</v>
@@ -4825,19 +4825,19 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>3016.01</v>
+        <v>3015.01</v>
       </c>
       <c r="E157" t="n">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="F157" t="n">
-        <v>89436</v>
+        <v>89434</v>
       </c>
       <c r="G157" t="n">
-        <v>16947.46</v>
+        <v>23302.54</v>
       </c>
       <c r="H157" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="158">
@@ -4943,7 +4943,7 @@
         <v>565</v>
       </c>
       <c r="F161" t="n">
-        <v>84965</v>
+        <v>84963</v>
       </c>
       <c r="G161" t="n">
         <v>31351.7</v>
@@ -4971,7 +4971,7 @@
         <v>884</v>
       </c>
       <c r="F162" t="n">
-        <v>66360</v>
+        <v>66355</v>
       </c>
       <c r="G162" t="n">
         <v>16097.45</v>
@@ -4993,13 +4993,13 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>962.5</v>
+        <v>961.22</v>
       </c>
       <c r="E163" t="n">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="F163" t="n">
-        <v>47679</v>
+        <v>47675</v>
       </c>
       <c r="G163" t="n">
         <v>5931.36</v>
@@ -5027,13 +5027,13 @@
         <v>147</v>
       </c>
       <c r="F164" t="n">
-        <v>63388</v>
+        <v>63385</v>
       </c>
       <c r="G164" t="n">
-        <v>3710.17</v>
+        <v>7117.8</v>
       </c>
       <c r="H164" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="165">
@@ -5083,7 +5083,7 @@
         <v>218</v>
       </c>
       <c r="F166" t="n">
-        <v>151053</v>
+        <v>151049</v>
       </c>
       <c r="G166" t="n">
         <v>3092.37</v>
@@ -5111,7 +5111,7 @@
         <v>216</v>
       </c>
       <c r="F167" t="n">
-        <v>44963</v>
+        <v>44962</v>
       </c>
       <c r="G167" t="n">
         <v>6774.58</v>
@@ -5139,7 +5139,7 @@
         <v>203</v>
       </c>
       <c r="F168" t="n">
-        <v>49685</v>
+        <v>49683</v>
       </c>
       <c r="G168" t="n">
         <v>7876.28</v>
@@ -5310,10 +5310,10 @@
         <v>38509</v>
       </c>
       <c r="G174" t="n">
-        <v>7875.440000000001</v>
+        <v>8976.290000000001</v>
       </c>
       <c r="H174" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="175">
@@ -5363,7 +5363,7 @@
         <v>270</v>
       </c>
       <c r="F176" t="n">
-        <v>30578</v>
+        <v>30573</v>
       </c>
       <c r="G176" t="n">
         <v>4574.57</v>
@@ -5839,13 +5839,13 @@
         <v>1589</v>
       </c>
       <c r="F193" t="n">
-        <v>171254</v>
+        <v>171253</v>
       </c>
       <c r="G193" t="n">
-        <v>110734.72</v>
+        <v>113022.01</v>
       </c>
       <c r="H193" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="194">
@@ -5895,7 +5895,7 @@
         <v>532</v>
       </c>
       <c r="F195" t="n">
-        <v>115195</v>
+        <v>115193</v>
       </c>
       <c r="G195" t="n">
         <v>11177.1</v>
@@ -5945,13 +5945,13 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>278.44</v>
+        <v>270.91</v>
       </c>
       <c r="E197" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F197" t="n">
-        <v>5365</v>
+        <v>5363</v>
       </c>
       <c r="G197" t="n">
         <v>0</v>
@@ -5979,7 +5979,7 @@
         <v>132</v>
       </c>
       <c r="F198" t="n">
-        <v>13507</v>
+        <v>13505</v>
       </c>
       <c r="G198" t="n">
         <v>10676.28</v>
@@ -6007,7 +6007,7 @@
         <v>27</v>
       </c>
       <c r="F199" t="n">
-        <v>3290</v>
+        <v>3288</v>
       </c>
       <c r="G199" t="n">
         <v>0</v>
@@ -6063,7 +6063,7 @@
         <v>3</v>
       </c>
       <c r="F201" t="n">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="G201" t="n">
         <v>1821.19</v>
@@ -6091,7 +6091,7 @@
         <v>36</v>
       </c>
       <c r="F202" t="n">
-        <v>5998</v>
+        <v>5997</v>
       </c>
       <c r="G202" t="n">
         <v>4211.01</v>
@@ -6147,7 +6147,7 @@
         <v>58</v>
       </c>
       <c r="F204" t="n">
-        <v>7736</v>
+        <v>7734</v>
       </c>
       <c r="G204" t="n">
         <v>0</v>
@@ -6175,7 +6175,7 @@
         <v>18</v>
       </c>
       <c r="F205" t="n">
-        <v>1423</v>
+        <v>1421</v>
       </c>
       <c r="G205" t="n">
         <v>0</v>
@@ -6203,13 +6203,13 @@
         <v>296</v>
       </c>
       <c r="F206" t="n">
-        <v>28971</v>
+        <v>28970</v>
       </c>
       <c r="G206" t="n">
-        <v>8133.9</v>
+        <v>12200.85</v>
       </c>
       <c r="H206" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="207">
@@ -6231,7 +6231,7 @@
         <v>911</v>
       </c>
       <c r="F207" t="n">
-        <v>62516</v>
+        <v>62514</v>
       </c>
       <c r="G207" t="n">
         <v>21476.26</v>
@@ -6315,7 +6315,7 @@
         <v>16</v>
       </c>
       <c r="F210" t="n">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="G210" t="n">
         <v>0</v>
@@ -6343,7 +6343,7 @@
         <v>31</v>
       </c>
       <c r="F211" t="n">
-        <v>4365</v>
+        <v>4364</v>
       </c>
       <c r="G211" t="n">
         <v>1694.07</v>
@@ -6399,7 +6399,7 @@
         <v>24</v>
       </c>
       <c r="F213" t="n">
-        <v>3470</v>
+        <v>3469</v>
       </c>
       <c r="G213" t="n">
         <v>6522.89</v>
@@ -6427,7 +6427,7 @@
         <v>460</v>
       </c>
       <c r="F214" t="n">
-        <v>46806</v>
+        <v>46805</v>
       </c>
       <c r="G214" t="n">
         <v>2837.28</v>
@@ -6455,7 +6455,7 @@
         <v>36</v>
       </c>
       <c r="F215" t="n">
-        <v>8425</v>
+        <v>8423</v>
       </c>
       <c r="G215" t="n">
         <v>9150.84</v>
@@ -6483,7 +6483,7 @@
         <v>142</v>
       </c>
       <c r="F216" t="n">
-        <v>16428</v>
+        <v>16426</v>
       </c>
       <c r="G216" t="n">
         <v>16012.71</v>
@@ -6511,7 +6511,7 @@
         <v>535</v>
       </c>
       <c r="F217" t="n">
-        <v>44640</v>
+        <v>44638</v>
       </c>
       <c r="G217" t="n">
         <v>34508.4</v>
@@ -6539,7 +6539,7 @@
         <v>34</v>
       </c>
       <c r="F218" t="n">
-        <v>1469</v>
+        <v>1468</v>
       </c>
       <c r="G218" t="n">
         <v>12370.33</v>
@@ -6567,7 +6567,7 @@
         <v>6</v>
       </c>
       <c r="F219" t="n">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="G219" t="n">
         <v>0</v>
@@ -6595,7 +6595,7 @@
         <v>3</v>
       </c>
       <c r="F220" t="n">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="G220" t="n">
         <v>0</v>
@@ -6651,7 +6651,7 @@
         <v>11</v>
       </c>
       <c r="F222" t="n">
-        <v>1550</v>
+        <v>1548</v>
       </c>
       <c r="G222" t="n">
         <v>0</v>
@@ -6679,7 +6679,7 @@
         <v>20</v>
       </c>
       <c r="F223" t="n">
-        <v>2837</v>
+        <v>2836</v>
       </c>
       <c r="G223" t="n">
         <v>0</v>
@@ -6707,7 +6707,7 @@
         <v>7</v>
       </c>
       <c r="F224" t="n">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="G224" t="n">
         <v>0</v>
@@ -6735,7 +6735,7 @@
         <v>9</v>
       </c>
       <c r="F225" t="n">
-        <v>1943</v>
+        <v>1941</v>
       </c>
       <c r="G225" t="n">
         <v>4083.9</v>
@@ -6763,13 +6763,13 @@
         <v>467</v>
       </c>
       <c r="F226" t="n">
-        <v>38652</v>
+        <v>38650</v>
       </c>
       <c r="G226" t="n">
-        <v>19300.89</v>
+        <v>19808.52</v>
       </c>
       <c r="H226" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="227">
@@ -6819,7 +6819,7 @@
         <v>93</v>
       </c>
       <c r="F228" t="n">
-        <v>12502</v>
+        <v>12500</v>
       </c>
       <c r="G228" t="n">
         <v>1355.08</v>
@@ -6847,7 +6847,7 @@
         <v>74</v>
       </c>
       <c r="F229" t="n">
-        <v>13522</v>
+        <v>13520</v>
       </c>
       <c r="G229" t="n">
         <v>0</v>
@@ -6875,7 +6875,7 @@
         <v>73</v>
       </c>
       <c r="F230" t="n">
-        <v>8134</v>
+        <v>8131</v>
       </c>
       <c r="G230" t="n">
         <v>0</v>
@@ -6931,7 +6931,7 @@
         <v>307</v>
       </c>
       <c r="F232" t="n">
-        <v>32421</v>
+        <v>32419</v>
       </c>
       <c r="G232" t="n">
         <v>5931.36</v>
@@ -6987,7 +6987,7 @@
         <v>12</v>
       </c>
       <c r="F234" t="n">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="G234" t="n">
         <v>0</v>
@@ -7015,7 +7015,7 @@
         <v>10</v>
       </c>
       <c r="F235" t="n">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="G235" t="n">
         <v>0</v>
@@ -7071,7 +7071,7 @@
         <v>47</v>
       </c>
       <c r="F237" t="n">
-        <v>8276</v>
+        <v>8273</v>
       </c>
       <c r="G237" t="n">
         <v>5337.29</v>
@@ -7099,7 +7099,7 @@
         <v>300</v>
       </c>
       <c r="F238" t="n">
-        <v>20525</v>
+        <v>20523</v>
       </c>
       <c r="G238" t="n">
         <v>52272.13</v>
@@ -7127,7 +7127,7 @@
         <v>7</v>
       </c>
       <c r="F239" t="n">
-        <v>2040</v>
+        <v>2039</v>
       </c>
       <c r="G239" t="n">
         <v>0</v>
@@ -7155,13 +7155,13 @@
         <v>381</v>
       </c>
       <c r="F240" t="n">
-        <v>34692</v>
+        <v>34691</v>
       </c>
       <c r="G240" t="n">
-        <v>36262.71</v>
+        <v>40160.17</v>
       </c>
       <c r="H240" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="241">
@@ -7183,7 +7183,7 @@
         <v>16</v>
       </c>
       <c r="F241" t="n">
-        <v>1758</v>
+        <v>1757</v>
       </c>
       <c r="G241" t="n">
         <v>0</v>
@@ -7211,7 +7211,7 @@
         <v>9</v>
       </c>
       <c r="F242" t="n">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G242" t="n">
         <v>2541.53</v>
@@ -7239,13 +7239,13 @@
         <v>11</v>
       </c>
       <c r="F243" t="n">
-        <v>1347</v>
+        <v>1346</v>
       </c>
       <c r="G243" t="n">
         <v>1609.32</v>
       </c>
       <c r="H243" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="244">
@@ -7267,7 +7267,7 @@
         <v>52</v>
       </c>
       <c r="F244" t="n">
-        <v>5934</v>
+        <v>5932</v>
       </c>
       <c r="G244" t="n">
         <v>34440.67</v>
@@ -7295,7 +7295,7 @@
         <v>479</v>
       </c>
       <c r="F245" t="n">
-        <v>25153</v>
+        <v>25151</v>
       </c>
       <c r="G245" t="n">
         <v>28635.58</v>
@@ -7323,7 +7323,7 @@
         <v>269</v>
       </c>
       <c r="F246" t="n">
-        <v>17741</v>
+        <v>17739</v>
       </c>
       <c r="G246" t="n">
         <v>12286.44</v>
@@ -7351,7 +7351,7 @@
         <v>402</v>
       </c>
       <c r="F247" t="n">
-        <v>31049</v>
+        <v>31048</v>
       </c>
       <c r="G247" t="n">
         <v>8473.73</v>
@@ -7379,7 +7379,7 @@
         <v>93</v>
       </c>
       <c r="F248" t="n">
-        <v>11149</v>
+        <v>11147</v>
       </c>
       <c r="G248" t="n">
         <v>7202.54</v>
@@ -7413,7 +7413,7 @@
         <v>44401.69</v>
       </c>
       <c r="H249" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="250">
@@ -7435,7 +7435,7 @@
         <v>10</v>
       </c>
       <c r="F250" t="n">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G250" t="n">
         <v>2880.51</v>
@@ -7463,7 +7463,7 @@
         <v>105</v>
       </c>
       <c r="F251" t="n">
-        <v>8033</v>
+        <v>8031</v>
       </c>
       <c r="G251" t="n">
         <v>0</v>
@@ -7491,7 +7491,7 @@
         <v>122</v>
       </c>
       <c r="F252" t="n">
-        <v>8104</v>
+        <v>8102</v>
       </c>
       <c r="G252" t="n">
         <v>6094.88</v>
@@ -7519,7 +7519,7 @@
         <v>7</v>
       </c>
       <c r="F253" t="n">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="G253" t="n">
         <v>1439.83</v>
@@ -7547,7 +7547,7 @@
         <v>24</v>
       </c>
       <c r="F254" t="n">
-        <v>1580</v>
+        <v>1579</v>
       </c>
       <c r="G254" t="n">
         <v>2129.66</v>
@@ -7575,7 +7575,7 @@
         <v>303</v>
       </c>
       <c r="F255" t="n">
-        <v>15475</v>
+        <v>15473</v>
       </c>
       <c r="G255" t="n">
         <v>12794.07</v>
@@ -7603,7 +7603,7 @@
         <v>276</v>
       </c>
       <c r="F256" t="n">
-        <v>29672</v>
+        <v>29670</v>
       </c>
       <c r="G256" t="n">
         <v>24317.82</v>
@@ -7631,7 +7631,7 @@
         <v>333</v>
       </c>
       <c r="F257" t="n">
-        <v>36319</v>
+        <v>36318</v>
       </c>
       <c r="G257" t="n">
         <v>18472.03</v>
@@ -7715,7 +7715,7 @@
         <v>312</v>
       </c>
       <c r="F260" t="n">
-        <v>47288</v>
+        <v>47284</v>
       </c>
       <c r="G260" t="n">
         <v>9461.01</v>
@@ -7771,7 +7771,7 @@
         <v>459</v>
       </c>
       <c r="F262" t="n">
-        <v>112244</v>
+        <v>112241</v>
       </c>
       <c r="G262" t="n">
         <v>19990.66</v>
@@ -7827,13 +7827,13 @@
         <v>124</v>
       </c>
       <c r="F264" t="n">
-        <v>25977</v>
+        <v>25975</v>
       </c>
       <c r="G264" t="n">
         <v>7242.37</v>
       </c>
       <c r="H264" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="265">
@@ -7883,7 +7883,7 @@
         <v>23</v>
       </c>
       <c r="F266" t="n">
-        <v>13120</v>
+        <v>13118</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
@@ -7911,7 +7911,7 @@
         <v>39</v>
       </c>
       <c r="F267" t="n">
-        <v>13195</v>
+        <v>13194</v>
       </c>
       <c r="G267" t="n">
         <v>3896.61</v>
@@ -7939,7 +7939,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>7617</v>
+        <v>7614</v>
       </c>
       <c r="G268" t="n">
         <v>4828.81</v>
@@ -7995,7 +7995,7 @@
         <v>120</v>
       </c>
       <c r="F270" t="n">
-        <v>32370</v>
+        <v>32368</v>
       </c>
       <c r="G270" t="n">
         <v>12706.78</v>
@@ -8051,7 +8051,7 @@
         <v>27</v>
       </c>
       <c r="F272" t="n">
-        <v>3652</v>
+        <v>3651</v>
       </c>
       <c r="G272" t="n">
         <v>5421.19</v>
@@ -8079,7 +8079,7 @@
         <v>417</v>
       </c>
       <c r="F273" t="n">
-        <v>55575</v>
+        <v>55573</v>
       </c>
       <c r="G273" t="n">
         <v>16900.85</v>
@@ -8303,13 +8303,13 @@
         <v>532</v>
       </c>
       <c r="F7" t="n">
-        <v>135892</v>
+        <v>135873</v>
       </c>
       <c r="G7" t="n">
         <v>27532.21</v>
       </c>
       <c r="H7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -8325,19 +8325,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2345.5</v>
+        <v>2344.97</v>
       </c>
       <c r="E8" t="n">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F8" t="n">
-        <v>122171</v>
+        <v>122170</v>
       </c>
       <c r="G8" t="n">
         <v>22365.25</v>
       </c>
       <c r="H8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -8502,10 +8502,10 @@
         <v>203845</v>
       </c>
       <c r="G14" t="n">
-        <v>36390.67</v>
+        <v>50963.55</v>
       </c>
       <c r="H14" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -8835,7 +8835,7 @@
         <v>222</v>
       </c>
       <c r="F26" t="n">
-        <v>37618</v>
+        <v>37617</v>
       </c>
       <c r="G26" t="n">
         <v>7626.27</v>
@@ -9025,19 +9025,19 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>4288.88</v>
+        <v>4288.18</v>
       </c>
       <c r="E33" t="n">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="F33" t="n">
-        <v>224914</v>
+        <v>224913</v>
       </c>
       <c r="G33" t="n">
         <v>35707.6</v>
       </c>
       <c r="H33" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="34">
@@ -9053,10 +9053,10 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1579.22</v>
+        <v>1578.52</v>
       </c>
       <c r="E34" t="n">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="F34" t="n">
         <v>83923</v>
@@ -9090,10 +9090,10 @@
         <v>64483</v>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>7202.54</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -9471,7 +9471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9534,19 +9534,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21839</v>
+        <v>15440</v>
       </c>
       <c r="E2" t="n">
-        <v>131</v>
+        <v>93</v>
       </c>
       <c r="F2" t="n">
-        <v>2058.54</v>
+        <v>1455.363518592124</v>
       </c>
       <c r="G2" t="n">
-        <v>12327.11</v>
+        <v>8715.121485942542</v>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -9576,10 +9576,10 @@
         <v>3591.95</v>
       </c>
       <c r="G3" t="n">
-        <v>6506.78</v>
+        <v>11082.2</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -9591,25 +9591,25 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Audio Array_SB_Branded_KT</t>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B0FJ8TSQK1</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>874</v>
+        <v>6399</v>
       </c>
       <c r="E4" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="F4" t="n">
-        <v>114.6095896787848</v>
+        <v>603.1764814078761</v>
       </c>
       <c r="G4" t="n">
-        <v>3854.505867995846</v>
+        <v>3611.98851405746</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -9629,23 +9629,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>B0BPLZ5CGV</t>
+          <t>B0B4DPX2J2</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>4662</v>
+        <v>874</v>
       </c>
       <c r="E5" t="n">
-        <v>114</v>
+        <v>21</v>
       </c>
       <c r="F5" t="n">
-        <v>611.3525288694003</v>
+        <v>114.6095896787848</v>
       </c>
       <c r="G5" t="n">
-        <v>20560.77433437844</v>
+        <v>4048.789674140955</v>
       </c>
       <c r="H5" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -9662,23 +9662,23 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>B0D3M1B4Z8</t>
+          <t>B0BPLZ5CGV</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1133</v>
+        <v>4662</v>
       </c>
       <c r="E6" t="n">
-        <v>28</v>
+        <v>114</v>
       </c>
       <c r="F6" t="n">
-        <v>148.5808846293487</v>
+        <v>611.3525288694003</v>
       </c>
       <c r="G6" t="n">
-        <v>4997.015461628957</v>
+        <v>21597.12649773647</v>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -9695,23 +9695,23 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>B0DN6MNS1X</t>
+          <t>B0D3M1B4Z8</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1619</v>
+        <v>1133</v>
       </c>
       <c r="E7" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="F7" t="n">
-        <v>212.2768747590112</v>
+        <v>148.5808846293487</v>
       </c>
       <c r="G7" t="n">
-        <v>7139.214630221187</v>
+        <v>5248.886704402813</v>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -9728,23 +9728,23 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>B0FG88HVQ8</t>
+          <t>B0DN6MNS1X</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>647</v>
+        <v>1619</v>
       </c>
       <c r="E8" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="F8" t="n">
-        <v>84.88539557340553</v>
+        <v>212.2768747590112</v>
       </c>
       <c r="G8" t="n">
-        <v>2854.833144956333</v>
+        <v>7499.061998145266</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -9761,23 +9761,23 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>B0FJ8TSQK1</t>
+          <t>B0FG88HVQ8</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1020</v>
+        <v>647</v>
       </c>
       <c r="E9" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F9" t="n">
-        <v>133.7185370397994</v>
+        <v>84.88539557340553</v>
       </c>
       <c r="G9" t="n">
-        <v>4497.170674149397</v>
+        <v>2998.729111989772</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -9794,20 +9794,20 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>B0G53H49BS</t>
+          <t>B0FJ8TSQK1</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>906</v>
+        <v>1020</v>
       </c>
       <c r="E10" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F10" t="n">
-        <v>118.8561894502501</v>
+        <v>133.7185370397994</v>
       </c>
       <c r="G10" t="n">
-        <v>3997.325886669838</v>
+        <v>4723.847572662514</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
@@ -9822,28 +9822,28 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Audio Array_Studio Headphones_SB_KT_Phrase</t>
+          <t>Audio Array_SB_Branded_KT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>B0FQBXS6Y2</t>
+          <t>B0G53H49BS</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>42738</v>
+        <v>906</v>
       </c>
       <c r="E11" t="n">
-        <v>111</v>
+        <v>22</v>
       </c>
       <c r="F11" t="n">
-        <v>1518.98</v>
+        <v>118.8561894502501</v>
       </c>
       <c r="G11" t="n">
-        <v>1270.34</v>
+        <v>4198.808440922217</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -9855,28 +9855,28 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AudioArray - Conference Mic - SB - AD</t>
+          <t>Audio Array_Studio Headphones_SB_KT_Phrase</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>B0B4K87PR4</t>
+          <t>B0FQBXS6Y2</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>23619</v>
+        <v>42738</v>
       </c>
       <c r="E12" t="n">
-        <v>57</v>
+        <v>111</v>
       </c>
       <c r="F12" t="n">
-        <v>530.7689699357554</v>
+        <v>1518.98</v>
       </c>
       <c r="G12" t="n">
-        <v>7517.35305222117</v>
+        <v>1270.34</v>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -9893,23 +9893,23 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>B0B4KC7VBM</t>
+          <t>B0B4K87PR4</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>15528</v>
+        <v>23619</v>
       </c>
       <c r="E13" t="n">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="F13" t="n">
-        <v>348.9491407327997</v>
+        <v>530.7689699357554</v>
       </c>
       <c r="G13" t="n">
-        <v>4942.214102070015</v>
+        <v>7517.35305222117</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -9926,23 +9926,23 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>B0CKHVHVQ1</t>
+          <t>B0B4KC7VBM</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>69892</v>
+        <v>15528</v>
       </c>
       <c r="E14" t="n">
-        <v>168</v>
+        <v>37</v>
       </c>
       <c r="F14" t="n">
-        <v>1570.63414819278</v>
+        <v>348.9491407327997</v>
       </c>
       <c r="G14" t="n">
-        <v>22245.10488860892</v>
+        <v>4942.214102070015</v>
       </c>
       <c r="H14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -9959,23 +9959,23 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>B0H3LHF2WW</t>
+          <t>B0CKHVHVQ1</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8088</v>
+        <v>69892</v>
       </c>
       <c r="E15" t="n">
-        <v>19</v>
+        <v>168</v>
       </c>
       <c r="F15" t="n">
-        <v>181.7477411386643</v>
+        <v>1570.63414819278</v>
       </c>
       <c r="G15" t="n">
-        <v>2574.117957099893</v>
+        <v>22245.10488860892</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -9987,28 +9987,28 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AudioArray - Podcast Mic  SB - KT</t>
+          <t>AudioArray - Conference Mic - SB - AD</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B0H3LHF2WW</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2254</v>
+        <v>8088</v>
       </c>
       <c r="E16" t="n">
         <v>19</v>
       </c>
       <c r="F16" t="n">
-        <v>163.197577520488</v>
+        <v>181.7477411386643</v>
       </c>
       <c r="G16" t="n">
-        <v>2447.95105288787</v>
+        <v>2574.117957099893</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -10025,23 +10025,23 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>B0FJS57732</t>
+          <t>B0B4DPX2J2</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4776</v>
+        <v>2254</v>
       </c>
       <c r="E17" t="n">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="F17" t="n">
-        <v>345.8172143717479</v>
+        <v>163.197577520488</v>
       </c>
       <c r="G17" t="n">
-        <v>5187.231495037324</v>
+        <v>2447.95105288787</v>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -10058,23 +10058,23 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>B0FTVQQVDC</t>
+          <t>B0FJS57732</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>25142</v>
+        <v>4775</v>
       </c>
       <c r="E18" t="n">
-        <v>214</v>
+        <v>41</v>
       </c>
       <c r="F18" t="n">
-        <v>1820.545208107764</v>
+        <v>345.8172143717479</v>
       </c>
       <c r="G18" t="n">
-        <v>27308.0374520748</v>
+        <v>5187.231495037324</v>
       </c>
       <c r="H18" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -10086,28 +10086,28 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AudioArray_Audio Mixers_SB_Collection</t>
+          <t>AudioArray - Podcast Mic  SB - KT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>B0CH4VCD6R</t>
+          <t>B0FTVQQVDC</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1390</v>
+        <v>25140</v>
       </c>
       <c r="E19" t="n">
-        <v>15</v>
+        <v>214</v>
       </c>
       <c r="F19" t="n">
-        <v>108.8263589631862</v>
+        <v>1820.545208107764</v>
       </c>
       <c r="G19" t="n">
-        <v>632.5782374875852</v>
+        <v>27308.0374520748</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -10124,23 +10124,23 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>B0G53H49BS</t>
+          <t>B0CH4VCD6R</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>21253</v>
+        <v>1389</v>
       </c>
       <c r="E20" t="n">
-        <v>230</v>
+        <v>15</v>
       </c>
       <c r="F20" t="n">
-        <v>1664.520504576765</v>
+        <v>108.8263589631862</v>
       </c>
       <c r="G20" t="n">
-        <v>9675.408210645954</v>
+        <v>632.5782374875853</v>
       </c>
       <c r="H20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -10157,23 +10157,23 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>B0G53M9258</t>
+          <t>B0G53H49BS</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>15184</v>
+        <v>21252</v>
       </c>
       <c r="E21" t="n">
-        <v>164</v>
+        <v>230</v>
       </c>
       <c r="F21" t="n">
-        <v>1189.172114632869</v>
+        <v>1664.520504576765</v>
       </c>
       <c r="G21" t="n">
-        <v>6912.336381651014</v>
+        <v>9675.408210645955</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -10190,23 +10190,23 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>B0GCP1J2HC</t>
+          <t>B0G53M9258</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>21512</v>
+        <v>15183</v>
       </c>
       <c r="E22" t="n">
-        <v>233</v>
+        <v>164</v>
       </c>
       <c r="F22" t="n">
-        <v>1684.741974178844</v>
+        <v>1189.172114632869</v>
       </c>
       <c r="G22" t="n">
-        <v>9792.950152893782</v>
+        <v>6912.336381651015</v>
       </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -10223,25 +10223,58 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>B0GCP1J2HC</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>21511</v>
+      </c>
+      <c r="E23" t="n">
+        <v>233</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1684.741974178844</v>
+      </c>
+      <c r="G23" t="n">
+        <v>9792.950152893782</v>
+      </c>
+      <c r="H23" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>AudioArray_Audio Mixers_SB_Collection</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>B0GXP97CZG</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>9616</v>
-      </c>
-      <c r="E23" t="n">
+      <c r="D24" t="n">
+        <v>9615</v>
+      </c>
+      <c r="E24" t="n">
         <v>104</v>
       </c>
-      <c r="F23" t="n">
-        <v>753.069047648336</v>
-      </c>
-      <c r="G23" t="n">
-        <v>4377.387017321666</v>
-      </c>
-      <c r="H23" t="n">
+      <c r="F24" t="n">
+        <v>753.0690476483361</v>
+      </c>
+      <c r="G24" t="n">
+        <v>4377.387017321667</v>
+      </c>
+      <c r="H24" t="n">
         <v>1</v>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Audio Array</t>
         </is>

</xml_diff>